<commit_message>
Project Empty Project is saved.
</commit_message>
<xml_diff>
--- a/Empty Project/Main.xlsx
+++ b/Empty Project/Main.xlsx
@@ -13,8 +13,47 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+  <si>
+    <t>Datatype Class extends Bank</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Default</t>
+  </si>
+  <si>
+    <t>Mandatory</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>strField</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datatype Class </t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -39,7 +78,7 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -344,9 +383,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="B2:G4"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+    </row>
+    <row r="3">
+      <c r="B3" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E4" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:G2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>